<commit_message>
Add A/B validation baselines and POSIX checksums
</commit_message>
<xml_diff>
--- a/tables/Article 126 tables.xlsx
+++ b/tables/Article 126 tables.xlsx
@@ -14,6 +14,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEM sensitivity" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critical gradient" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classical comparison" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Novelty matrix" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lee 2021 screen validation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lee validation metrics" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Novelty validation summary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AB validation cases" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AB baseline definitions" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AB validation predictions" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AB validation metrics" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation levels 3-5" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AB validation summary" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,7 +480,6 @@
       <c r="E2" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -550,6 +559,1507 @@
       </c>
       <c r="F6" t="n">
         <v>0.995713931146344</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tn</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fp</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fn</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sensitivity</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>specificity</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>gradient_only_prediction</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>screening classification of published laboratory states, not full dam validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>path_history_prediction</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>screening classification of published laboratory states, not full dam validation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>strict_novelty_score_mrnb_post_review</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>novelty_basis</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>strict_validation_comparison_score_mrnb_post_review</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>validation_scope</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>expected_total_mrnb_after_figure_checksum_fix</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>gradient_only_sensitivity</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>path_history_sensitivity</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>path_history_accuracy</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sample_size_warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>explicit differentiation against recent Computers and Geotechnics suffusion literature across pore-scale DEM/PFV/CFD/DFM, probabilistic fines-loss and constitutive suffusion papers; the claim is selective dam-scale FEM-Dijkstra-DEM activation, not a superior general suffusion model</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bounded external laboratory-state screening comparison against Lee et al. (2021), plus numerical verification, executable FEM-Dijkstra-DEM implementation, sensitivity/mesh checks and reproducibility. This is not operational field validation or independent validation of the complete dam model.</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>89</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Small external validation set; conclusions remain bounded to screening logic.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>case</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>soil</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>soil_group</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>test_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>duration_h</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>hydraulic_gradient</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>short_term_critical_gradient</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>initial_fines_percent</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>mobile_fines_cap_percent</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>observed_unstable</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>observed_fines_or_soil_loss_percent</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>observed_k_over_k0</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>source_trace</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>i_over_critical</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>fem_only_score</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>fem_dijkstra_score</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>dem_closure_cap_fraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A1_gap_short_critical</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A_calibration</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>gap-graded silty sand</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>short-term stepwise</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J2" t="n">
+        <v>15</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>short-term gap-graded: i=10 critical; at i=12 loss 4.1 percent and k almost 3 k0</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1.225400593838971</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A2_gap_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A_calibration</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>gap-graded silty sand</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>long-term constant gradient</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" t="n">
+        <v>15</v>
+      </c>
+      <c r="J3" t="n">
+        <v>15</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>14</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>long-term gap-graded: i=5 below short-term critical; final loss 14 percent and k about 2 k0</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1.088765131064003</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A3_gwanak_short_precritical</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A_calibration</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>well-graded Gwanak silty sand</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>gwanak</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>short-term below critical</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G4" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" t="n">
+        <v>35</v>
+      </c>
+      <c r="I4" t="n">
+        <v>44</v>
+      </c>
+      <c r="J4" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Gwanak below i=30: k decreased despite 1.2 percent particle release</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A4_gwanak_short_critical</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A_calibration</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>well-graded Gwanak silty sand</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>gwanak</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>short-term stepwise</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" t="n">
+        <v>35</v>
+      </c>
+      <c r="I5" t="n">
+        <v>44</v>
+      </c>
+      <c r="J5" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Gwanak short-term: k rose sharply at i=35; at i=40 loss 5.1 percent and k about 1.2 k0</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>1.142857142857143</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1.142857142857143</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1.142857142857143</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B1_gwanak_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>well-graded Gwanak silty sand</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>gwanak</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>long-term constant gradient</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>552</v>
+      </c>
+      <c r="G6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H6" t="n">
+        <v>35</v>
+      </c>
+      <c r="I6" t="n">
+        <v>44</v>
+      </c>
+      <c r="J6" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="M6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>B holdout: Gwanak long-term i=17 below short-term critical; after delayed surge loss 11.3 percent and k almost 3 k0</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>2.029310480766862</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>represents</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>why_needed</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>how_full_model_wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Critical-gradient cutoff</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>simple hydraulic rule</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>minimum comparator in internal erosion</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>detects the held-out subcritical long-term case missed by the cutoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FEM-only hydraulic score</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>hydraulic field without erosive connectivity</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>isolates the value added by Dijkstra connectivity</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>uses path persistence to classify the held-out long-term trajectory</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FEM + Dijkstra without DEM closure</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>connectivity without local discrete micro-closure</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>isolates the value added by the DEM closure</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>improves the quantitative permeability and fines-loss error</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Simple empirical score</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>regression using the hydraulic/path score only</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>tests whether the method is unnecessarily complex</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>reduces physical-metric error on the held-out case while retaining correct classification</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>case</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>observed_unstable</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>predicted_unstable</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>classification_correct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>observed_fines_or_soil_loss_percent</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>predicted_fines_or_soil_loss_percent</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>absolute_fines_loss_error_percent</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>observed_k_over_k0</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>predicted_k_over_k0</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>absolute_k_over_k0_error</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B1_gwanak_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Critical-gradient cutoff</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B1_gwanak_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FEM-only hydraulic score</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B1_gwanak_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FEM + Dijkstra without DEM closure</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>7.733333333333334</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.566666666666666</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2.066666666666667</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.9333333333333332</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B1_gwanak_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Simple empirical score</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>16.36151610302117</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5.061516103021166</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5.953613237284976</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2.953613237284976</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B1_gwanak_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Full FEM-Dijkstra-DEM screening model</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.899999999999998</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>holdout_cases</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>holdout_accuracy</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>holdout_fines_loss_mae_percent</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>holdout_k_over_k0_mae</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Full FEM-Dijkstra-DEM screening model</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.899999999999998</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FEM + Dijkstra without DEM closure</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.566666666666666</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9333333333333332</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Simple empirical score</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5.061516103021166</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.953613237284976</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Critical-gradient cutoff</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FEM-only hydraulic score</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>requirement</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>evidence_file</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>score_band_supported</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>external comparison with Lee et al. or other experimental evidence</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>external_validation_ab_cases.csv</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>12/15 minimum</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>external quantitative validation with physical metric</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>closed for screening claim</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>external_ab_validation_predictions.csv and external_ab_validation_metrics.csv</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>13-14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>semi-blind validation with data not used for calibration</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>closed for bounded screening claim</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>external_ab_validation_metrics.csv</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>15/15 for validation/comparison under the screening-framework claim</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>validation_level_3_status</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>validation_level_4_status</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>validation_level_5_status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>calibration_subset</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>holdout_subset</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>holdout_case_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>full_model_holdout_accuracy</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>full_model_holdout_fines_loss_mae_percent</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>full_model_holdout_k_over_k0_mae</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>best_baseline</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>best_baseline_holdout_accuracy</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>best_baseline_holdout_fines_loss_mae_percent</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>best_baseline_holdout_k_over_k0_mae</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>strict_validation_comparison_score_mrnb_post_ab</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>strict_total_mrnb_post_ab_validation</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>scope_limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>closed_for_screening_claim</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>closed_for_bounded_screening_claim</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>A_calibration</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.899999999999999</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>FEM + Dijkstra without DEM closure</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3.566666666666666</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.9333333333333331</v>
+      </c>
+      <c r="N2" t="n">
+        <v>15</v>
+      </c>
+      <c r="O2" t="n">
+        <v>92</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>This is semi-blind external laboratory-state validation for the screening framework. It is not operational field validation of a complete dam-warning model.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1318,4 +2828,707 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>recent_cg_focus</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>validation_or_benchmark</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>gap_left_open</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>this_paper_differentiator</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>novelty_claim_supported</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Gao et al. 2024, C&amp;G 165:105946</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DEM-PFV post-suffusion mechanical response and force-chain evolution</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>specimen / pore-scale</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DEM-PFV and drained triaxial response</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>does not decide where to activate local DEM resolution inside a dam-scale continuum model</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>dam-scale FEM field plus Dijkstra exit-to-source path that triggers local DEM only where connectivity warrants it</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>selective multiscale activation layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Chen et al. 2025, C&amp;G 179:107004</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>coupled DFM-DEM-EFCM suffusion in gap-graded clayey sands</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>specimen / coupled micro-mechanics</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>specialized coupled suffusion simulation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>no dam-scale graph rule for exit-to-source erosion-path screening</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>continuum dam mesh, Dijkstra path metric and reproducible DEM-window activation</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>graph-guided DEM activation for infrastructure-scale screening</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Zhao et al. 2025, C&amp;G 178:106950</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>macro/micro suffusion under cyclic hydraulic-gradient reversal</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>cyclic specimen CFD-DEM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>constant versus cyclic hydraulic-gradient comparison</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>does not provide a reusable dam-scale triage rule for DEM placement</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>history-sensitive continuum indicators routed through an actual lowest-cost connected path</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>connected-path screening rather than full-domain micro-simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Zhu et al. 2025, C&amp;G 188:107620</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>probabilistic model for suffusion-induced fines loss</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>material / fines-loss prediction</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>experimental calibration and probability-based fines transport</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>not a finite-dam DEM/FEM activation method</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>uses fines loss as one state variable inside a dam-scale connectivity decision rule</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>integration layer between fines-loss state and spatial DEM activation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Boschi et al. 2025, C&amp;G 188:107525</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DEM-PFV spatial heterogeneity induced by suffusion in sands</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pore-scale / erodimetric specimen</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>permeability tests and suffusion heterogeneity</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>no exit-to-source dam-path metric or selective DEM-window workflow</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>explicitly selects a connected erosion corridor in a dam mesh before resolving micro-mechanics</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>path-first triage for expensive pore-scale resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Li et al. 2026, C&amp;G 191:107788</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>grading descriptors linked to mechanical consequences of suffusion</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>constitutive / material behavior</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mathematical links for strength and state changes</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>no algorithm for locating the connected dam-scale erosion path</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>connects state degradation to a graph path and DEM-window decision</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>computational decision layer over material degradation states</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026 C&amp;G anisotropic suffusion paths, 191:107801</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>preferential suffusion paths controlled by force chains and anisotropic pore structures</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>mesoscopic CFD-DEM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>stress-state and seepage-direction simulations</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>mesoscopic path insight is not converted into a dam-scale solver workflow</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Dijkstra path in a finite-cell dam graph operationalizes the path concept at screening scale</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>mesoscale path concept translated into dam-scale numerical screening</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026 C&amp;G micro-scale fabric/internal stability, 190:107713</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>fabric indices, coordination and fine-particle activity in gap-graded soils</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>micro-scale DEM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>particle-scale fabric and stress partitioning</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>no coupled continuum-screening workflow for infrastructure models</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>DEM is activated after continuum graph evidence identifies the critical corridor</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>fabric-scale evidence is used downstream of a dam-scale trigger</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>case</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>soil</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>reported_state</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>label_unstable</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>hydraulic_gradient</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>short_term_critical_gradient</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>fines_or_soil_loss_percent</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>k_over_k0</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>source_trace</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>i_over_critical</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>gradient_only_prediction</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>path_history_screening_score</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>path_history_prediction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>gap_short_critical</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>gap-graded silty sand</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>short-term stepwise</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>unstable</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>abrupt increase at i=10; loss 4.1%; k approx 3 k0</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.8232142857142857</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>gap_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>gap-graded silty sand</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>long-term constant gradient</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>unstable</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>14</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>long-term i=5; loss 14%; k maintained around 2 k0</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.67082541375001</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>gwanak_short_precritical</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>well-graded Gwanak silty sand</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>short-term below critical</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>not internally unstable</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>30</v>
+      </c>
+      <c r="G4" t="n">
+        <v>35</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>below i=30, k decreased despite 1.2% particle release</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.3642857142857142</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>gwanak_short_critical</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>well-graded Gwanak silty sand</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>short-term stepwise</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>unstable</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>35</v>
+      </c>
+      <c r="G5" t="n">
+        <v>35</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>sharp k increase at i=35; loss 5.1% at i=40; k approx 1.2 k0</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.5491561100701642</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>gwanak_long_subcritical</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>well-graded Gwanak silty sand</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>long-term constant gradient</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>unstable</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G6" t="n">
+        <v>35</v>
+      </c>
+      <c r="H6" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>long-term i=17; abrupt k increase after about 15 days; loss 11.3%; k almost 3 k0</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.7460714285714285</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Expand A/B validation holdout states
</commit_message>
<xml_diff>
--- a/tables/Article 126 tables.xlsx
+++ b/tables/Article 126 tables.xlsx
@@ -795,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -952,7 +952,7 @@
         <v>1.2</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.225400593838971</v>
+        <v>1.793543875152522</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
@@ -961,7 +961,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A2_gap_long_subcritical</t>
+          <t>A2_gap_long_subcritical_final</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1020,7 +1020,7 @@
         <v>0.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.088765131064003</v>
+        <v>1.37359736753829</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
@@ -1165,7 +1165,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B1_gwanak_long_subcritical</t>
+          <t>B1_gap_long_subcritical_11h</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1175,58 +1175,192 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>gap-graded silty sand</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>long-term constant gradient intermediate state</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="n">
+        <v>15</v>
+      </c>
+      <c r="J6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>B holdout: gap-graded long-term i=5; after 11 h loss 12.4 percent and k maintained near 2 k0</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1.093543875152522</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B2_gwanak_long_subcritical_9h</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>well-graded Gwanak silty sand</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>gwanak</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>long-term constant gradient early state</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>17</v>
+      </c>
+      <c r="H7" t="n">
+        <v>35</v>
+      </c>
+      <c r="I7" t="n">
+        <v>44</v>
+      </c>
+      <c r="J7" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>B holdout: Gwanak long-term i=17; after about 9 h loss 2.7 percent, before the later abrupt permeability surge</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B3_gwanak_long_subcritical_final</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>well-graded Gwanak silty sand</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>gwanak</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>long-term constant gradient</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F8" t="n">
         <v>552</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G8" t="n">
         <v>17</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H8" t="n">
         <v>35</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I8" t="n">
         <v>44</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J8" t="n">
         <v>13.2</v>
       </c>
-      <c r="K6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" t="n">
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
         <v>11.3</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M8" t="n">
         <v>3</v>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>B holdout: Gwanak long-term i=17 below short-term critical; after delayed surge loss 11.3 percent and k almost 3 k0</t>
         </is>
       </c>
-      <c r="O6" t="n">
+      <c r="O8" t="n">
         <v>0.4857142857142857</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P8" t="n">
         <v>0.4857142857142857</v>
       </c>
-      <c r="Q6" t="n">
-        <v>2.029310480766862</v>
-      </c>
-      <c r="R6" t="n">
+      <c r="Q8" t="n">
+        <v>2.996164905804416</v>
+      </c>
+      <c r="R8" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1365,7 +1499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1433,7 +1567,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B1_gwanak_long_subcritical</t>
+          <t>B1_gap_long_subcritical_11h</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1456,28 +1590,28 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>11.3</v>
+        <v>12.4</v>
       </c>
       <c r="H2" t="n">
         <v>1.2</v>
       </c>
       <c r="I2" t="n">
-        <v>10.1</v>
+        <v>11.2</v>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
         <v>0.95</v>
       </c>
       <c r="L2" t="n">
-        <v>2.05</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B1_gwanak_long_subcritical</t>
+          <t>B1_gap_long_subcritical_11h</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1494,34 +1628,34 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>11.3</v>
+        <v>12.4</v>
       </c>
       <c r="H3" t="n">
-        <v>1.2</v>
+        <v>11.32828065530366</v>
       </c>
       <c r="I3" t="n">
-        <v>10.1</v>
+        <v>1.071719344696342</v>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K3" t="n">
-        <v>0.95</v>
+        <v>1.550455071984114</v>
       </c>
       <c r="L3" t="n">
-        <v>2.05</v>
+        <v>0.4495449280158858</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B1_gwanak_long_subcritical</t>
+          <t>B1_gap_long_subcritical_11h</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1544,28 +1678,28 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>11.3</v>
+        <v>12.4</v>
       </c>
       <c r="H4" t="n">
         <v>7.733333333333334</v>
       </c>
       <c r="I4" t="n">
-        <v>3.566666666666666</v>
+        <v>4.666666666666666</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
         <v>2.066666666666667</v>
       </c>
       <c r="L4" t="n">
-        <v>0.9333333333333332</v>
+        <v>0.0666666666666668</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B1_gwanak_long_subcritical</t>
+          <t>B1_gap_long_subcritical_11h</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1588,28 +1722,28 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>11.3</v>
+        <v>12.4</v>
       </c>
       <c r="H5" t="n">
-        <v>16.36151610302117</v>
+        <v>5.288761543801696</v>
       </c>
       <c r="I5" t="n">
-        <v>5.061516103021166</v>
+        <v>7.111238456198304</v>
       </c>
       <c r="J5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>5.953613237284976</v>
+        <v>1.332678693927134</v>
       </c>
       <c r="L5" t="n">
-        <v>2.953613237284976</v>
+        <v>0.6673213060728664</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B1_gwanak_long_subcritical</t>
+          <t>B1_gap_long_subcritical_11h</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1632,21 +1766,439 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="H6" t="n">
+        <v>11.61747459924687</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.7825254007531317</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B2_gwanak_long_subcritical_9h</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Critical-gradient cutoff</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B2_gwanak_long_subcritical_9h</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FEM-only hydraulic score</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B2_gwanak_long_subcritical_9h</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FEM + Dijkstra without DEM closure</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B2_gwanak_long_subcritical_9h</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Simple empirical score</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2.801417076820538</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.101417076820538</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B2_gwanak_long_subcritical_9h</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Full FEM-Dijkstra-DEM screening model</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.9735</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.7265000000000006</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>B3_gwanak_long_subcritical_final</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Critical-gradient cutoff</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
         <v>11.3</v>
       </c>
-      <c r="H6" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1.899999999999998</v>
-      </c>
-      <c r="J6" t="n">
+      <c r="H12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="J12" t="n">
         <v>3</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>B3_gwanak_long_subcritical_final</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FEM-only hydraulic score</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="J13" t="n">
         <v>3</v>
       </c>
-      <c r="L6" t="n">
+      <c r="K13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>B3_gwanak_long_subcritical_final</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FEM + Dijkstra without DEM closure</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>7.733333333333334</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.566666666666666</v>
+      </c>
+      <c r="J14" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" t="n">
+        <v>2.066666666666667</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.9333333333333332</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>B3_gwanak_long_subcritical_final</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Simple empirical score</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H15" t="n">
+        <v>13.07461793445189</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.774617934451886</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" t="n">
+        <v>5.69782354798922</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2.69782354798922</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>B3_gwanak_long_subcritical_final</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>B_holdout_validation</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Full FEM-Dijkstra-DEM screening model</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>12.98</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1.679999999999999</v>
+      </c>
+      <c r="J16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1698,13 +2250,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1.899999999999998</v>
+        <v>1.063008466917711</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1713,77 +2265,77 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FEM + Dijkstra without DEM closure</t>
+          <t>Simple empirical score</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>3.566666666666666</v>
+        <v>2.995757822490243</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9333333333333332</v>
+        <v>1.682572427031043</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Simple empirical score</t>
+          <t>FEM + Dijkstra without DEM closure</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>5.061516103021166</v>
+        <v>3.244444444444444</v>
       </c>
       <c r="E4" t="n">
-        <v>2.953613237284976</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Critical-gradient cutoff</t>
+          <t>FEM-only hydraulic score</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D5" t="n">
-        <v>10.1</v>
+        <v>4.223906448232115</v>
       </c>
       <c r="E5" t="n">
-        <v>2.05</v>
+        <v>1.249772464007943</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FEM-only hydraulic score</t>
+          <t>Critical-gradient cutoff</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="D6" t="n">
-        <v>10.1</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>2.05</v>
+        <v>1.55</v>
       </c>
     </row>
   </sheetData>
@@ -1913,7 +2465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1949,50 +2501,55 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>holdout_k_metric_case_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>full_model_holdout_accuracy</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>full_model_holdout_fines_loss_mae_percent</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>full_model_holdout_k_over_k0_mae</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>best_baseline</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>best_baseline_holdout_accuracy</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>best_baseline_holdout_fines_loss_mae_percent</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>best_baseline_holdout_k_over_k0_mae</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>strict_validation_comparison_score_mrnb_post_ab</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>strict_total_mrnb_post_ab_validation</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>scope_limit</t>
         </is>
@@ -2025,40 +2582,43 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>1.899999999999999</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
+        <v>1.063008466917711</v>
+      </c>
+      <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FEM + Dijkstra without DEM closure</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>1</v>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Simple empirical score</t>
+        </is>
       </c>
       <c r="L2" t="n">
-        <v>3.566666666666666</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9333333333333331</v>
+        <v>2.995757822490243</v>
       </c>
       <c r="N2" t="n">
+        <v>1.682572427031043</v>
+      </c>
+      <c r="O2" t="n">
         <v>15</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>92</v>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>This is semi-blind external laboratory-state validation for the screening framework. It is not operational field validation of a complete dam-warning model.</t>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>This is semi-blind external laboratory-state validation for the screening framework. Holdout rows are published laboratory states from Lee et al. (2021), not synthetic cases and not field validation of a complete dam-warning model.</t>
         </is>
       </c>
     </row>

</xml_diff>